<commit_message>
anpassung Tabellen + html Tabellen
</commit_message>
<xml_diff>
--- a/Webseite/build/html/Tabellen_Untersuchungsgebeite/Charakterisierung_Messszenarien.xlsx
+++ b/Webseite/build/html/Tabellen_Untersuchungsgebeite/Charakterisierung_Messszenarien.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\(0)_Bachelorarbeit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\(0)_Bachelorarbeit\Digitaler_Anhang\Digitaler_Anhang-Galileo_HAS\Webseite\build\html\Tabellen_Untersuchungsgebeite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A27A05-A56E-485A-A070-E606DC0E82F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230FB1D4-C9DE-4406-AED1-E2B99BA6A952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -229,10 +229,10 @@
     <t>Ø PDop</t>
   </si>
   <si>
-    <t>Konvergiert [%]</t>
-  </si>
-  <si>
     <t>Punkt 1, 23,  34, 41, 42, 46, 74, 87, 90, 99, 100,  133, 268,  311, 349, 402, 496, 503, 504, 511 haben 0 Sat.empf</t>
+  </si>
+  <si>
+    <t>Konvergierend [%]</t>
   </si>
 </sst>
 </file>
@@ -268,12 +268,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -559,6 +560,7 @@
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="14" max="14" width="10.28515625" customWidth="1"/>
     <col min="15" max="15" width="16.28515625" customWidth="1"/>
     <col min="16" max="16" width="16.42578125" customWidth="1"/>
@@ -596,7 +598,7 @@
         <v>56</v>
       </c>
       <c r="J1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K1" t="s">
         <v>57</v>
@@ -642,7 +644,7 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E2">
@@ -704,7 +706,7 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E3">
@@ -769,7 +771,7 @@
       <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E4">
@@ -834,7 +836,7 @@
       <c r="C5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E5">
@@ -896,7 +898,7 @@
       <c r="C6" t="s">
         <v>30</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>31</v>
       </c>
       <c r="E6">
@@ -961,7 +963,7 @@
       <c r="C7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E7">
@@ -1026,7 +1028,7 @@
       <c r="C8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E8">
@@ -1088,7 +1090,7 @@
       <c r="C9" t="s">
         <v>42</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E9">
@@ -1153,7 +1155,7 @@
       <c r="C10" t="s">
         <v>46</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E10">
@@ -1218,7 +1220,7 @@
       <c r="C11" t="s">
         <v>50</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E11">
@@ -1270,7 +1272,7 @@
         <v>16</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>